<commit_message>
remove target_cash and replace with reuired sale for deployment
</commit_message>
<xml_diff>
--- a/data/exports/prod-portfolio_intelligence.xlsx
+++ b/data/exports/prod-portfolio_intelligence.xlsx
@@ -15382,7 +15382,7 @@
         <v>0.4922</v>
       </c>
       <c r="D40">
-        <v>0.2634</v>
+        <v>0.2638</v>
       </c>
       <c r="E40">
         <v>0</v>
@@ -15782,7 +15782,7 @@
         <v>0.4619</v>
       </c>
       <c r="D48">
-        <v>0.3267</v>
+        <v>0.327</v>
       </c>
       <c r="E48">
         <v>0</v>

</xml_diff>